<commit_message>
Update test files with column width preservation applied
Regenerated sample_complex.xlsx and added width_test files
used to verify column width/row height conversion.

https://claude.ai/code/session_0179fduQDX21vgHwbjCgDbza
</commit_message>
<xml_diff>
--- a/sample_complex.xlsx
+++ b/sample_complex.xlsx
@@ -418,7 +418,7 @@
   <dimension ref="A1:F28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="12.75" customHeight="1">
       <c r="A1" t="inlineStr">
         <is>
           <t>請求書</t>
@@ -430,7 +430,7 @@
       <c r="E1" t="inlineStr"/>
       <c r="F1" t="inlineStr"/>
     </row>
-    <row r="2">
+    <row r="2" ht="12.75" customHeight="1">
       <c r="A2" t="inlineStr">
         <is>
           <t>請求番号</t>
@@ -446,7 +446,7 @@
       <c r="E2" t="inlineStr"/>
       <c r="F2" t="inlineStr"/>
     </row>
-    <row r="3">
+    <row r="3" ht="12.75" customHeight="1">
       <c r="A3" t="inlineStr">
         <is>
           <t>発行日</t>
@@ -462,7 +462,7 @@
       <c r="E3" t="inlineStr"/>
       <c r="F3" t="inlineStr"/>
     </row>
-    <row r="4">
+    <row r="4" ht="12.75" customHeight="1">
       <c r="A4" t="inlineStr">
         <is>
           <t>支払期限</t>
@@ -486,7 +486,7 @@
       <c r="E5" t="inlineStr"/>
       <c r="F5" t="inlineStr"/>
     </row>
-    <row r="6">
+    <row r="6" ht="12.75" customHeight="1">
       <c r="A6" t="inlineStr">
         <is>
           <t>請求先</t>
@@ -502,7 +502,7 @@
       <c r="E6" t="inlineStr"/>
       <c r="F6" t="inlineStr"/>
     </row>
-    <row r="7">
+    <row r="7" ht="12.75" customHeight="1">
       <c r="A7" t="inlineStr">
         <is>
           <t>会社名</t>
@@ -526,7 +526,7 @@
       </c>
       <c r="F7" t="inlineStr"/>
     </row>
-    <row r="8">
+    <row r="8" ht="12.75" customHeight="1">
       <c r="A8" t="inlineStr">
         <is>
           <t>担当者</t>
@@ -550,7 +550,7 @@
       </c>
       <c r="F8" t="inlineStr"/>
     </row>
-    <row r="9">
+    <row r="9" ht="12.75" customHeight="1">
       <c r="A9" t="inlineStr">
         <is>
           <t>住所</t>
@@ -574,7 +574,7 @@
       </c>
       <c r="F9" t="inlineStr"/>
     </row>
-    <row r="10">
+    <row r="10" ht="12.75" customHeight="1">
       <c r="A10" t="inlineStr"/>
       <c r="B10" t="inlineStr"/>
       <c r="C10" t="inlineStr"/>
@@ -598,7 +598,7 @@
       <c r="E11" t="inlineStr"/>
       <c r="F11" t="inlineStr"/>
     </row>
-    <row r="12">
+    <row r="12" ht="12.75" customHeight="1">
       <c r="A12" t="inlineStr">
         <is>
           <t>No.</t>
@@ -630,7 +630,7 @@
         </is>
       </c>
     </row>
-    <row r="13">
+    <row r="13" ht="12.75" customHeight="1">
       <c r="A13" t="n">
         <v>1</v>
       </c>
@@ -654,7 +654,7 @@
         <v>500000</v>
       </c>
     </row>
-    <row r="14">
+    <row r="14" ht="12.75" customHeight="1">
       <c r="A14" t="n">
         <v>2</v>
       </c>
@@ -678,7 +678,7 @@
         <v>400000</v>
       </c>
     </row>
-    <row r="15">
+    <row r="15" ht="12.75" customHeight="1">
       <c r="A15" t="n">
         <v>3</v>
       </c>
@@ -702,7 +702,7 @@
         <v>1200000</v>
       </c>
     </row>
-    <row r="16">
+    <row r="16" ht="12.75" customHeight="1">
       <c r="A16" t="n">
         <v>4</v>
       </c>
@@ -726,7 +726,7 @@
         <v>600000</v>
       </c>
     </row>
-    <row r="17">
+    <row r="17" ht="12.75" customHeight="1">
       <c r="A17" t="n">
         <v>5</v>
       </c>
@@ -750,7 +750,7 @@
         <v>150000</v>
       </c>
     </row>
-    <row r="18">
+    <row r="18" ht="12.75" customHeight="1">
       <c r="A18" t="n">
         <v>6</v>
       </c>
@@ -774,7 +774,7 @@
         <v>80000</v>
       </c>
     </row>
-    <row r="19">
+    <row r="19" ht="12.75" customHeight="1">
       <c r="A19" t="n">
         <v>7</v>
       </c>
@@ -806,7 +806,7 @@
       <c r="E20" t="inlineStr"/>
       <c r="F20" t="inlineStr"/>
     </row>
-    <row r="21">
+    <row r="21" ht="12.75" customHeight="1">
       <c r="A21" t="inlineStr"/>
       <c r="B21" t="inlineStr"/>
       <c r="C21" t="inlineStr"/>
@@ -820,7 +820,7 @@
         <v>3080000</v>
       </c>
     </row>
-    <row r="22">
+    <row r="22" ht="12.75" customHeight="1">
       <c r="A22" t="inlineStr"/>
       <c r="B22" t="inlineStr"/>
       <c r="C22" t="inlineStr"/>
@@ -834,7 +834,7 @@
         <v>308000</v>
       </c>
     </row>
-    <row r="23">
+    <row r="23" ht="12.75" customHeight="1">
       <c r="A23" t="inlineStr"/>
       <c r="B23" t="inlineStr"/>
       <c r="C23" t="inlineStr"/>
@@ -856,7 +856,7 @@
       <c r="E24" t="inlineStr"/>
       <c r="F24" t="inlineStr"/>
     </row>
-    <row r="25">
+    <row r="25" ht="12.75" customHeight="1">
       <c r="A25" t="inlineStr">
         <is>
           <t>備考</t>
@@ -868,7 +868,7 @@
       <c r="E25" t="inlineStr"/>
       <c r="F25" t="inlineStr"/>
     </row>
-    <row r="26">
+    <row r="26" ht="12.75" customHeight="1">
       <c r="A26" t="inlineStr">
         <is>
           <t>・お振込先：〇〇銀行 △△支店 普通 1234567 カ）テストカイハツ</t>
@@ -880,7 +880,7 @@
       <c r="E26" t="inlineStr"/>
       <c r="F26" t="inlineStr"/>
     </row>
-    <row r="27">
+    <row r="27" ht="12.75" customHeight="1">
       <c r="A27" t="inlineStr">
         <is>
           <t>・振込手数料はご負担ください。</t>
@@ -892,7 +892,7 @@
       <c r="E27" t="inlineStr"/>
       <c r="F27" t="inlineStr"/>
     </row>
-    <row r="28">
+    <row r="28" ht="12.75" customHeight="1">
       <c r="A28" t="inlineStr">
         <is>
           <t>・本請求書に関するお問い合わせは担当者までご連絡ください。</t>
@@ -918,7 +918,7 @@
   <dimension ref="A1:H23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="12.75" customHeight="1">
       <c r="A1" t="inlineStr">
         <is>
           <t>月次売上明細レポート</t>
@@ -932,7 +932,7 @@
       <c r="G1" t="inlineStr"/>
       <c r="H1" t="inlineStr"/>
     </row>
-    <row r="2">
+    <row r="2" ht="12.75" customHeight="1">
       <c r="A2" t="inlineStr">
         <is>
           <t>対象期間</t>
@@ -950,7 +950,7 @@
       <c r="G2" t="inlineStr"/>
       <c r="H2" t="inlineStr"/>
     </row>
-    <row r="3">
+    <row r="3" ht="12.75" customHeight="1">
       <c r="A3" t="inlineStr">
         <is>
           <t>作成日</t>
@@ -978,7 +978,7 @@
       <c r="G4" t="inlineStr"/>
       <c r="H4" t="inlineStr"/>
     </row>
-    <row r="5">
+    <row r="5" ht="12.75" customHeight="1">
       <c r="A5" t="inlineStr">
         <is>
           <t>月</t>
@@ -1020,7 +1020,7 @@
         </is>
       </c>
     </row>
-    <row r="6">
+    <row r="6" ht="12.75" customHeight="1">
       <c r="A6" t="inlineStr">
         <is>
           <t>2024/01</t>
@@ -1054,7 +1054,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="7">
+    <row r="7" ht="12.75" customHeight="1">
       <c r="A7" t="inlineStr">
         <is>
           <t>2024/01</t>
@@ -1088,7 +1088,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="8">
+    <row r="8" ht="12.75" customHeight="1">
       <c r="A8" t="inlineStr">
         <is>
           <t>2024/01</t>
@@ -1122,7 +1122,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="9">
+    <row r="9" ht="12.75" customHeight="1">
       <c r="A9" t="inlineStr">
         <is>
           <t>2024/02</t>
@@ -1156,7 +1156,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="10">
+    <row r="10" ht="12.75" customHeight="1">
       <c r="A10" t="inlineStr">
         <is>
           <t>2024/02</t>
@@ -1190,7 +1190,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="11">
+    <row r="11" ht="12.75" customHeight="1">
       <c r="A11" t="inlineStr">
         <is>
           <t>2024/02</t>
@@ -1224,7 +1224,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="12">
+    <row r="12" ht="12.75" customHeight="1">
       <c r="A12" t="inlineStr">
         <is>
           <t>2024/03</t>
@@ -1258,7 +1258,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="13">
+    <row r="13" ht="12.75" customHeight="1">
       <c r="A13" t="inlineStr">
         <is>
           <t>2024/03</t>
@@ -1292,7 +1292,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="14">
+    <row r="14" ht="12.75" customHeight="1">
       <c r="A14" t="inlineStr">
         <is>
           <t>2024/03</t>
@@ -1326,7 +1326,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="15">
+    <row r="15" ht="12.75" customHeight="1">
       <c r="A15" t="inlineStr">
         <is>
           <t>2024/03</t>
@@ -1360,7 +1360,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="16">
+    <row r="16" ht="12.75" customHeight="1">
       <c r="A16" t="inlineStr">
         <is>
           <t>合計</t>
@@ -1392,7 +1392,7 @@
       <c r="G17" t="inlineStr"/>
       <c r="H17" t="inlineStr"/>
     </row>
-    <row r="18">
+    <row r="18" ht="12.75" customHeight="1">
       <c r="A18" t="inlineStr">
         <is>
           <t>担当者別集計</t>
@@ -1406,7 +1406,7 @@
       <c r="G18" t="inlineStr"/>
       <c r="H18" t="inlineStr"/>
     </row>
-    <row r="19">
+    <row r="19" ht="12.75" customHeight="1">
       <c r="A19" t="inlineStr">
         <is>
           <t>担当者</t>
@@ -1428,7 +1428,7 @@
       <c r="G19" t="inlineStr"/>
       <c r="H19" t="inlineStr"/>
     </row>
-    <row r="20">
+    <row r="20" ht="12.75" customHeight="1">
       <c r="A20" t="inlineStr">
         <is>
           <t>佐藤 二郎</t>
@@ -1446,7 +1446,7 @@
       <c r="G20" t="inlineStr"/>
       <c r="H20" t="inlineStr"/>
     </row>
-    <row r="21">
+    <row r="21" ht="12.75" customHeight="1">
       <c r="A21" t="inlineStr">
         <is>
           <t>山本 四郎</t>
@@ -1464,7 +1464,7 @@
       <c r="G21" t="inlineStr"/>
       <c r="H21" t="inlineStr"/>
     </row>
-    <row r="22">
+    <row r="22" ht="12.75" customHeight="1">
       <c r="A22" t="inlineStr">
         <is>
           <t>田中 一郎</t>
@@ -1482,7 +1482,7 @@
       <c r="G22" t="inlineStr"/>
       <c r="H22" t="inlineStr"/>
     </row>
-    <row r="23">
+    <row r="23" ht="12.75" customHeight="1">
       <c r="A23" t="inlineStr">
         <is>
           <t>鈴木 三郎</t>
@@ -1514,7 +1514,7 @@
   <dimension ref="A1:F19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="12.75" customHeight="1">
       <c r="A1" t="inlineStr">
         <is>
           <t>経費精算書</t>
@@ -1526,7 +1526,7 @@
       <c r="E1" t="inlineStr"/>
       <c r="F1" t="inlineStr"/>
     </row>
-    <row r="2">
+    <row r="2" ht="12.75" customHeight="1">
       <c r="A2" t="inlineStr">
         <is>
           <t>申請者</t>
@@ -1542,7 +1542,7 @@
       <c r="E2" t="inlineStr"/>
       <c r="F2" t="inlineStr"/>
     </row>
-    <row r="3">
+    <row r="3" ht="12.75" customHeight="1">
       <c r="A3" t="inlineStr">
         <is>
           <t>所属</t>
@@ -1558,7 +1558,7 @@
       <c r="E3" t="inlineStr"/>
       <c r="F3" t="inlineStr"/>
     </row>
-    <row r="4">
+    <row r="4" ht="12.75" customHeight="1">
       <c r="A4" t="inlineStr">
         <is>
           <t>申請日</t>
@@ -1574,7 +1574,7 @@
       <c r="E4" t="inlineStr"/>
       <c r="F4" t="inlineStr"/>
     </row>
-    <row r="5">
+    <row r="5" ht="12.75" customHeight="1">
       <c r="A5" t="inlineStr">
         <is>
           <t>精算対象月</t>
@@ -1598,7 +1598,7 @@
       <c r="E6" t="inlineStr"/>
       <c r="F6" t="inlineStr"/>
     </row>
-    <row r="7">
+    <row r="7" ht="12.75" customHeight="1">
       <c r="A7" t="inlineStr">
         <is>
           <t>日付</t>
@@ -1630,7 +1630,7 @@
         </is>
       </c>
     </row>
-    <row r="8">
+    <row r="8" ht="12.75" customHeight="1">
       <c r="A8" t="inlineStr">
         <is>
           <t>2024/03/05</t>
@@ -1660,7 +1660,7 @@
         </is>
       </c>
     </row>
-    <row r="9">
+    <row r="9" ht="12.75" customHeight="1">
       <c r="A9" t="inlineStr">
         <is>
           <t>2024/03/07</t>
@@ -1690,7 +1690,7 @@
         </is>
       </c>
     </row>
-    <row r="10">
+    <row r="10" ht="12.75" customHeight="1">
       <c r="A10" t="inlineStr">
         <is>
           <t>2024/03/12</t>
@@ -1720,7 +1720,7 @@
         </is>
       </c>
     </row>
-    <row r="11">
+    <row r="11" ht="12.75" customHeight="1">
       <c r="A11" t="inlineStr">
         <is>
           <t>2024/03/14</t>
@@ -1750,7 +1750,7 @@
         </is>
       </c>
     </row>
-    <row r="12">
+    <row r="12" ht="12.75" customHeight="1">
       <c r="A12" t="inlineStr">
         <is>
           <t>2024/03/19</t>
@@ -1780,7 +1780,7 @@
         </is>
       </c>
     </row>
-    <row r="13">
+    <row r="13" ht="12.75" customHeight="1">
       <c r="A13" t="inlineStr">
         <is>
           <t>2024/03/19</t>
@@ -1810,7 +1810,7 @@
         </is>
       </c>
     </row>
-    <row r="14">
+    <row r="14" ht="12.75" customHeight="1">
       <c r="A14" t="inlineStr">
         <is>
           <t>2024/03/22</t>
@@ -1840,7 +1840,7 @@
         </is>
       </c>
     </row>
-    <row r="15">
+    <row r="15" ht="12.75" customHeight="1">
       <c r="A15" t="inlineStr">
         <is>
           <t>2024/03/28</t>
@@ -1870,7 +1870,7 @@
         </is>
       </c>
     </row>
-    <row r="16">
+    <row r="16" ht="12.75" customHeight="1">
       <c r="A16" t="inlineStr"/>
       <c r="B16" t="inlineStr"/>
       <c r="C16" t="inlineStr"/>
@@ -1892,7 +1892,7 @@
       <c r="E17" t="inlineStr"/>
       <c r="F17" t="inlineStr"/>
     </row>
-    <row r="18">
+    <row r="18" ht="12.75" customHeight="1">
       <c r="A18" t="inlineStr">
         <is>
           <t>承認欄</t>
@@ -1904,7 +1904,7 @@
       <c r="E18" t="inlineStr"/>
       <c r="F18" t="inlineStr"/>
     </row>
-    <row r="19">
+    <row r="19" ht="12.75" customHeight="1">
       <c r="A19" t="inlineStr">
         <is>
           <t>担当</t>

</xml_diff>

<commit_message>
Copy and verify font size, bold, italic during conversion
Read font info via xf_list/font_list with formatting_info=True.
Convert XLS height (twips) to points. Verify size within 0.5pt,
bold and italic exact match.

https://claude.ai/code/session_0179fduQDX21vgHwbjCgDbza
</commit_message>
<xml_diff>
--- a/sample_complex.xlsx
+++ b/sample_complex.xlsx
@@ -19,13 +19,16 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
     </font>
   </fonts>
   <fills count="2">
@@ -48,8 +51,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -419,490 +423,490 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1" ht="12.75" customHeight="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>請求書</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr"/>
-      <c r="C1" t="inlineStr"/>
-      <c r="D1" t="inlineStr"/>
-      <c r="E1" t="inlineStr"/>
-      <c r="F1" t="inlineStr"/>
+      <c r="B1" s="1" t="inlineStr"/>
+      <c r="C1" s="1" t="inlineStr"/>
+      <c r="D1" s="1" t="inlineStr"/>
+      <c r="E1" s="1" t="inlineStr"/>
+      <c r="F1" s="1" t="inlineStr"/>
     </row>
     <row r="2" ht="12.75" customHeight="1">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="1" t="inlineStr">
         <is>
           <t>請求番号</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B2" s="1" t="inlineStr">
         <is>
           <t>INV-2024-00123</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr"/>
-      <c r="D2" t="inlineStr"/>
-      <c r="E2" t="inlineStr"/>
-      <c r="F2" t="inlineStr"/>
+      <c r="C2" s="1" t="inlineStr"/>
+      <c r="D2" s="1" t="inlineStr"/>
+      <c r="E2" s="1" t="inlineStr"/>
+      <c r="F2" s="1" t="inlineStr"/>
     </row>
     <row r="3" ht="12.75" customHeight="1">
-      <c r="A3" t="inlineStr">
+      <c r="A3" s="1" t="inlineStr">
         <is>
           <t>発行日</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B3" s="1" t="inlineStr">
         <is>
           <t>2024/03/31</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr"/>
-      <c r="D3" t="inlineStr"/>
-      <c r="E3" t="inlineStr"/>
-      <c r="F3" t="inlineStr"/>
+      <c r="C3" s="1" t="inlineStr"/>
+      <c r="D3" s="1" t="inlineStr"/>
+      <c r="E3" s="1" t="inlineStr"/>
+      <c r="F3" s="1" t="inlineStr"/>
     </row>
     <row r="4" ht="12.75" customHeight="1">
-      <c r="A4" t="inlineStr">
+      <c r="A4" s="1" t="inlineStr">
         <is>
           <t>支払期限</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="B4" s="1" t="inlineStr">
         <is>
           <t>2024/04/30</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr"/>
-      <c r="D4" t="inlineStr"/>
-      <c r="E4" t="inlineStr"/>
-      <c r="F4" t="inlineStr"/>
+      <c r="C4" s="1" t="inlineStr"/>
+      <c r="D4" s="1" t="inlineStr"/>
+      <c r="E4" s="1" t="inlineStr"/>
+      <c r="F4" s="1" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr"/>
-      <c r="B5" t="inlineStr"/>
-      <c r="C5" t="inlineStr"/>
-      <c r="D5" t="inlineStr"/>
-      <c r="E5" t="inlineStr"/>
-      <c r="F5" t="inlineStr"/>
+      <c r="A5" s="1" t="inlineStr"/>
+      <c r="B5" s="1" t="inlineStr"/>
+      <c r="C5" s="1" t="inlineStr"/>
+      <c r="D5" s="1" t="inlineStr"/>
+      <c r="E5" s="1" t="inlineStr"/>
+      <c r="F5" s="1" t="inlineStr"/>
     </row>
     <row r="6" ht="12.75" customHeight="1">
-      <c r="A6" t="inlineStr">
+      <c r="A6" s="1" t="inlineStr">
         <is>
           <t>請求先</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr"/>
-      <c r="C6" t="inlineStr"/>
-      <c r="D6" t="inlineStr">
+      <c r="B6" s="1" t="inlineStr"/>
+      <c r="C6" s="1" t="inlineStr"/>
+      <c r="D6" s="1" t="inlineStr">
         <is>
           <t>請求元</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr"/>
-      <c r="F6" t="inlineStr"/>
+      <c r="E6" s="1" t="inlineStr"/>
+      <c r="F6" s="1" t="inlineStr"/>
     </row>
     <row r="7" ht="12.75" customHeight="1">
-      <c r="A7" t="inlineStr">
+      <c r="A7" s="1" t="inlineStr">
         <is>
           <t>会社名</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
+      <c r="B7" s="1" t="inlineStr">
         <is>
           <t>株式会社サンプル商事</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr"/>
-      <c r="D7" t="inlineStr">
+      <c r="C7" s="1" t="inlineStr"/>
+      <c r="D7" s="1" t="inlineStr">
         <is>
           <t>会社名</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr">
+      <c r="E7" s="1" t="inlineStr">
         <is>
           <t>株式会社テスト開発</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr"/>
+      <c r="F7" s="1" t="inlineStr"/>
     </row>
     <row r="8" ht="12.75" customHeight="1">
-      <c r="A8" t="inlineStr">
+      <c r="A8" s="1" t="inlineStr">
         <is>
           <t>担当者</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
+      <c r="B8" s="1" t="inlineStr">
         <is>
           <t>山田 太郎 様</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr"/>
-      <c r="D8" t="inlineStr">
+      <c r="C8" s="1" t="inlineStr"/>
+      <c r="D8" s="1" t="inlineStr">
         <is>
           <t>担当者</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr">
+      <c r="E8" s="1" t="inlineStr">
         <is>
           <t>鈴木 花子</t>
         </is>
       </c>
-      <c r="F8" t="inlineStr"/>
+      <c r="F8" s="1" t="inlineStr"/>
     </row>
     <row r="9" ht="12.75" customHeight="1">
-      <c r="A9" t="inlineStr">
+      <c r="A9" s="1" t="inlineStr">
         <is>
           <t>住所</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
+      <c r="B9" s="1" t="inlineStr">
         <is>
           <t>〒100-0001 東京都千代田区千代田1-1-1</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr"/>
-      <c r="D9" t="inlineStr">
+      <c r="C9" s="1" t="inlineStr"/>
+      <c r="D9" s="1" t="inlineStr">
         <is>
           <t>電話</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr">
+      <c r="E9" s="1" t="inlineStr">
         <is>
           <t>03-1234-5678</t>
         </is>
       </c>
-      <c r="F9" t="inlineStr"/>
+      <c r="F9" s="1" t="inlineStr"/>
     </row>
     <row r="10" ht="12.75" customHeight="1">
-      <c r="A10" t="inlineStr"/>
-      <c r="B10" t="inlineStr"/>
-      <c r="C10" t="inlineStr"/>
-      <c r="D10" t="inlineStr">
+      <c r="A10" s="1" t="inlineStr"/>
+      <c r="B10" s="1" t="inlineStr"/>
+      <c r="C10" s="1" t="inlineStr"/>
+      <c r="D10" s="1" t="inlineStr">
         <is>
           <t>メール</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr">
+      <c r="E10" s="1" t="inlineStr">
         <is>
           <t>suzuki@test-dev.co.jp</t>
         </is>
       </c>
-      <c r="F10" t="inlineStr"/>
+      <c r="F10" s="1" t="inlineStr"/>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr"/>
-      <c r="B11" t="inlineStr"/>
-      <c r="C11" t="inlineStr"/>
-      <c r="D11" t="inlineStr"/>
-      <c r="E11" t="inlineStr"/>
-      <c r="F11" t="inlineStr"/>
+      <c r="A11" s="1" t="inlineStr"/>
+      <c r="B11" s="1" t="inlineStr"/>
+      <c r="C11" s="1" t="inlineStr"/>
+      <c r="D11" s="1" t="inlineStr"/>
+      <c r="E11" s="1" t="inlineStr"/>
+      <c r="F11" s="1" t="inlineStr"/>
     </row>
     <row r="12" ht="12.75" customHeight="1">
-      <c r="A12" t="inlineStr">
+      <c r="A12" s="1" t="inlineStr">
         <is>
           <t>No.</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr">
+      <c r="B12" s="1" t="inlineStr">
         <is>
           <t>品目</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr">
+      <c r="C12" s="1" t="inlineStr">
         <is>
           <t>数量</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr">
+      <c r="D12" s="1" t="inlineStr">
         <is>
           <t>単位</t>
         </is>
       </c>
-      <c r="E12" t="inlineStr">
+      <c r="E12" s="1" t="inlineStr">
         <is>
           <t>単価（円）</t>
         </is>
       </c>
-      <c r="F12" t="inlineStr">
+      <c r="F12" s="1" t="inlineStr">
         <is>
           <t>金額（円）</t>
         </is>
       </c>
     </row>
     <row r="13" ht="12.75" customHeight="1">
-      <c r="A13" t="n">
+      <c r="A13" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="B13" t="inlineStr">
+      <c r="B13" s="1" t="inlineStr">
         <is>
           <t>Webシステム開発（基本設計）</t>
         </is>
       </c>
-      <c r="C13" t="n">
+      <c r="C13" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="D13" t="inlineStr">
+      <c r="D13" s="1" t="inlineStr">
         <is>
           <t>式</t>
         </is>
       </c>
-      <c r="E13" t="n">
+      <c r="E13" s="1" t="n">
         <v>500000</v>
       </c>
-      <c r="F13" t="n">
+      <c r="F13" s="1" t="n">
         <v>500000</v>
       </c>
     </row>
     <row r="14" ht="12.75" customHeight="1">
-      <c r="A14" t="n">
+      <c r="A14" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="B14" t="inlineStr">
+      <c r="B14" s="1" t="inlineStr">
         <is>
           <t>Webシステム開発（詳細設計）</t>
         </is>
       </c>
-      <c r="C14" t="n">
+      <c r="C14" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="D14" t="inlineStr">
+      <c r="D14" s="1" t="inlineStr">
         <is>
           <t>式</t>
         </is>
       </c>
-      <c r="E14" t="n">
+      <c r="E14" s="1" t="n">
         <v>400000</v>
       </c>
-      <c r="F14" t="n">
+      <c r="F14" s="1" t="n">
         <v>400000</v>
       </c>
     </row>
     <row r="15" ht="12.75" customHeight="1">
-      <c r="A15" t="n">
+      <c r="A15" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="B15" t="inlineStr">
+      <c r="B15" s="1" t="inlineStr">
         <is>
           <t>Webシステム開発（実装）</t>
         </is>
       </c>
-      <c r="C15" t="n">
+      <c r="C15" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="D15" t="inlineStr">
+      <c r="D15" s="1" t="inlineStr">
         <is>
           <t>人月</t>
         </is>
       </c>
-      <c r="E15" t="n">
+      <c r="E15" s="1" t="n">
         <v>600000</v>
       </c>
-      <c r="F15" t="n">
+      <c r="F15" s="1" t="n">
         <v>1200000</v>
       </c>
     </row>
     <row r="16" ht="12.75" customHeight="1">
-      <c r="A16" t="n">
+      <c r="A16" s="1" t="n">
         <v>4</v>
       </c>
-      <c r="B16" t="inlineStr">
+      <c r="B16" s="1" t="inlineStr">
         <is>
           <t>Webシステム開発（テスト）</t>
         </is>
       </c>
-      <c r="C16" t="n">
+      <c r="C16" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="D16" t="inlineStr">
+      <c r="D16" s="1" t="inlineStr">
         <is>
           <t>人月</t>
         </is>
       </c>
-      <c r="E16" t="n">
+      <c r="E16" s="1" t="n">
         <v>600000</v>
       </c>
-      <c r="F16" t="n">
+      <c r="F16" s="1" t="n">
         <v>600000</v>
       </c>
     </row>
     <row r="17" ht="12.75" customHeight="1">
-      <c r="A17" t="n">
+      <c r="A17" s="1" t="n">
         <v>5</v>
       </c>
-      <c r="B17" t="inlineStr">
+      <c r="B17" s="1" t="inlineStr">
         <is>
           <t>サーバー構築・設定</t>
         </is>
       </c>
-      <c r="C17" t="n">
+      <c r="C17" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="D17" t="inlineStr">
+      <c r="D17" s="1" t="inlineStr">
         <is>
           <t>式</t>
         </is>
       </c>
-      <c r="E17" t="n">
+      <c r="E17" s="1" t="n">
         <v>150000</v>
       </c>
-      <c r="F17" t="n">
+      <c r="F17" s="1" t="n">
         <v>150000</v>
       </c>
     </row>
     <row r="18" ht="12.75" customHeight="1">
-      <c r="A18" t="n">
+      <c r="A18" s="1" t="n">
         <v>6</v>
       </c>
-      <c r="B18" t="inlineStr">
+      <c r="B18" s="1" t="inlineStr">
         <is>
           <t>ドキュメント作成</t>
         </is>
       </c>
-      <c r="C18" t="n">
+      <c r="C18" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="D18" t="inlineStr">
+      <c r="D18" s="1" t="inlineStr">
         <is>
           <t>式</t>
         </is>
       </c>
-      <c r="E18" t="n">
+      <c r="E18" s="1" t="n">
         <v>80000</v>
       </c>
-      <c r="F18" t="n">
+      <c r="F18" s="1" t="n">
         <v>80000</v>
       </c>
     </row>
     <row r="19" ht="12.75" customHeight="1">
-      <c r="A19" t="n">
+      <c r="A19" s="1" t="n">
         <v>7</v>
       </c>
-      <c r="B19" t="inlineStr">
+      <c r="B19" s="1" t="inlineStr">
         <is>
           <t>保守サポート（3ヶ月分）</t>
         </is>
       </c>
-      <c r="C19" t="n">
+      <c r="C19" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="D19" t="inlineStr">
+      <c r="D19" s="1" t="inlineStr">
         <is>
           <t>ヶ月</t>
         </is>
       </c>
-      <c r="E19" t="n">
+      <c r="E19" s="1" t="n">
         <v>50000</v>
       </c>
-      <c r="F19" t="n">
+      <c r="F19" s="1" t="n">
         <v>150000</v>
       </c>
     </row>
     <row r="20">
-      <c r="A20" t="inlineStr"/>
-      <c r="B20" t="inlineStr"/>
-      <c r="C20" t="inlineStr"/>
-      <c r="D20" t="inlineStr"/>
-      <c r="E20" t="inlineStr"/>
-      <c r="F20" t="inlineStr"/>
+      <c r="A20" s="1" t="inlineStr"/>
+      <c r="B20" s="1" t="inlineStr"/>
+      <c r="C20" s="1" t="inlineStr"/>
+      <c r="D20" s="1" t="inlineStr"/>
+      <c r="E20" s="1" t="inlineStr"/>
+      <c r="F20" s="1" t="inlineStr"/>
     </row>
     <row r="21" ht="12.75" customHeight="1">
-      <c r="A21" t="inlineStr"/>
-      <c r="B21" t="inlineStr"/>
-      <c r="C21" t="inlineStr"/>
-      <c r="D21" t="inlineStr"/>
-      <c r="E21" t="inlineStr">
+      <c r="A21" s="1" t="inlineStr"/>
+      <c r="B21" s="1" t="inlineStr"/>
+      <c r="C21" s="1" t="inlineStr"/>
+      <c r="D21" s="1" t="inlineStr"/>
+      <c r="E21" s="1" t="inlineStr">
         <is>
           <t>小計</t>
         </is>
       </c>
-      <c r="F21" t="n">
+      <c r="F21" s="1" t="n">
         <v>3080000</v>
       </c>
     </row>
     <row r="22" ht="12.75" customHeight="1">
-      <c r="A22" t="inlineStr"/>
-      <c r="B22" t="inlineStr"/>
-      <c r="C22" t="inlineStr"/>
-      <c r="D22" t="inlineStr"/>
-      <c r="E22" t="inlineStr">
+      <c r="A22" s="1" t="inlineStr"/>
+      <c r="B22" s="1" t="inlineStr"/>
+      <c r="C22" s="1" t="inlineStr"/>
+      <c r="D22" s="1" t="inlineStr"/>
+      <c r="E22" s="1" t="inlineStr">
         <is>
           <t>消費税（10%）</t>
         </is>
       </c>
-      <c r="F22" t="n">
+      <c r="F22" s="1" t="n">
         <v>308000</v>
       </c>
     </row>
     <row r="23" ht="12.75" customHeight="1">
-      <c r="A23" t="inlineStr"/>
-      <c r="B23" t="inlineStr"/>
-      <c r="C23" t="inlineStr"/>
-      <c r="D23" t="inlineStr"/>
-      <c r="E23" t="inlineStr">
+      <c r="A23" s="1" t="inlineStr"/>
+      <c r="B23" s="1" t="inlineStr"/>
+      <c r="C23" s="1" t="inlineStr"/>
+      <c r="D23" s="1" t="inlineStr"/>
+      <c r="E23" s="1" t="inlineStr">
         <is>
           <t>合計金額</t>
         </is>
       </c>
-      <c r="F23" t="n">
+      <c r="F23" s="1" t="n">
         <v>3388000</v>
       </c>
     </row>
     <row r="24">
-      <c r="A24" t="inlineStr"/>
-      <c r="B24" t="inlineStr"/>
-      <c r="C24" t="inlineStr"/>
-      <c r="D24" t="inlineStr"/>
-      <c r="E24" t="inlineStr"/>
-      <c r="F24" t="inlineStr"/>
+      <c r="A24" s="1" t="inlineStr"/>
+      <c r="B24" s="1" t="inlineStr"/>
+      <c r="C24" s="1" t="inlineStr"/>
+      <c r="D24" s="1" t="inlineStr"/>
+      <c r="E24" s="1" t="inlineStr"/>
+      <c r="F24" s="1" t="inlineStr"/>
     </row>
     <row r="25" ht="12.75" customHeight="1">
-      <c r="A25" t="inlineStr">
+      <c r="A25" s="1" t="inlineStr">
         <is>
           <t>備考</t>
         </is>
       </c>
-      <c r="B25" t="inlineStr"/>
-      <c r="C25" t="inlineStr"/>
-      <c r="D25" t="inlineStr"/>
-      <c r="E25" t="inlineStr"/>
-      <c r="F25" t="inlineStr"/>
+      <c r="B25" s="1" t="inlineStr"/>
+      <c r="C25" s="1" t="inlineStr"/>
+      <c r="D25" s="1" t="inlineStr"/>
+      <c r="E25" s="1" t="inlineStr"/>
+      <c r="F25" s="1" t="inlineStr"/>
     </row>
     <row r="26" ht="12.75" customHeight="1">
-      <c r="A26" t="inlineStr">
+      <c r="A26" s="1" t="inlineStr">
         <is>
           <t>・お振込先：〇〇銀行 △△支店 普通 1234567 カ）テストカイハツ</t>
         </is>
       </c>
-      <c r="B26" t="inlineStr"/>
-      <c r="C26" t="inlineStr"/>
-      <c r="D26" t="inlineStr"/>
-      <c r="E26" t="inlineStr"/>
-      <c r="F26" t="inlineStr"/>
+      <c r="B26" s="1" t="inlineStr"/>
+      <c r="C26" s="1" t="inlineStr"/>
+      <c r="D26" s="1" t="inlineStr"/>
+      <c r="E26" s="1" t="inlineStr"/>
+      <c r="F26" s="1" t="inlineStr"/>
     </row>
     <row r="27" ht="12.75" customHeight="1">
-      <c r="A27" t="inlineStr">
+      <c r="A27" s="1" t="inlineStr">
         <is>
           <t>・振込手数料はご負担ください。</t>
         </is>
       </c>
-      <c r="B27" t="inlineStr"/>
-      <c r="C27" t="inlineStr"/>
-      <c r="D27" t="inlineStr"/>
-      <c r="E27" t="inlineStr"/>
-      <c r="F27" t="inlineStr"/>
+      <c r="B27" s="1" t="inlineStr"/>
+      <c r="C27" s="1" t="inlineStr"/>
+      <c r="D27" s="1" t="inlineStr"/>
+      <c r="E27" s="1" t="inlineStr"/>
+      <c r="F27" s="1" t="inlineStr"/>
     </row>
     <row r="28" ht="12.75" customHeight="1">
-      <c r="A28" t="inlineStr">
+      <c r="A28" s="1" t="inlineStr">
         <is>
           <t>・本請求書に関するお問い合わせは担当者までご連絡ください。</t>
         </is>
       </c>
-      <c r="B28" t="inlineStr"/>
-      <c r="C28" t="inlineStr"/>
-      <c r="D28" t="inlineStr"/>
-      <c r="E28" t="inlineStr"/>
-      <c r="F28" t="inlineStr"/>
+      <c r="B28" s="1" t="inlineStr"/>
+      <c r="C28" s="1" t="inlineStr"/>
+      <c r="D28" s="1" t="inlineStr"/>
+      <c r="E28" s="1" t="inlineStr"/>
+      <c r="F28" s="1" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -919,586 +923,586 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1" ht="12.75" customHeight="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>月次売上明細レポート</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr"/>
-      <c r="C1" t="inlineStr"/>
-      <c r="D1" t="inlineStr"/>
-      <c r="E1" t="inlineStr"/>
-      <c r="F1" t="inlineStr"/>
-      <c r="G1" t="inlineStr"/>
-      <c r="H1" t="inlineStr"/>
+      <c r="B1" s="1" t="inlineStr"/>
+      <c r="C1" s="1" t="inlineStr"/>
+      <c r="D1" s="1" t="inlineStr"/>
+      <c r="E1" s="1" t="inlineStr"/>
+      <c r="F1" s="1" t="inlineStr"/>
+      <c r="G1" s="1" t="inlineStr"/>
+      <c r="H1" s="1" t="inlineStr"/>
     </row>
     <row r="2" ht="12.75" customHeight="1">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="1" t="inlineStr">
         <is>
           <t>対象期間</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B2" s="1" t="inlineStr">
         <is>
           <t>2024年1月〜3月</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr"/>
-      <c r="D2" t="inlineStr"/>
-      <c r="E2" t="inlineStr"/>
-      <c r="F2" t="inlineStr"/>
-      <c r="G2" t="inlineStr"/>
-      <c r="H2" t="inlineStr"/>
+      <c r="C2" s="1" t="inlineStr"/>
+      <c r="D2" s="1" t="inlineStr"/>
+      <c r="E2" s="1" t="inlineStr"/>
+      <c r="F2" s="1" t="inlineStr"/>
+      <c r="G2" s="1" t="inlineStr"/>
+      <c r="H2" s="1" t="inlineStr"/>
     </row>
     <row r="3" ht="12.75" customHeight="1">
-      <c r="A3" t="inlineStr">
+      <c r="A3" s="1" t="inlineStr">
         <is>
           <t>作成日</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B3" s="1" t="inlineStr">
         <is>
           <t>2024/03/31</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr"/>
-      <c r="D3" t="inlineStr"/>
-      <c r="E3" t="inlineStr"/>
-      <c r="F3" t="inlineStr"/>
-      <c r="G3" t="inlineStr"/>
-      <c r="H3" t="inlineStr"/>
+      <c r="C3" s="1" t="inlineStr"/>
+      <c r="D3" s="1" t="inlineStr"/>
+      <c r="E3" s="1" t="inlineStr"/>
+      <c r="F3" s="1" t="inlineStr"/>
+      <c r="G3" s="1" t="inlineStr"/>
+      <c r="H3" s="1" t="inlineStr"/>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr"/>
-      <c r="B4" t="inlineStr"/>
-      <c r="C4" t="inlineStr"/>
-      <c r="D4" t="inlineStr"/>
-      <c r="E4" t="inlineStr"/>
-      <c r="F4" t="inlineStr"/>
-      <c r="G4" t="inlineStr"/>
-      <c r="H4" t="inlineStr"/>
+      <c r="A4" s="1" t="inlineStr"/>
+      <c r="B4" s="1" t="inlineStr"/>
+      <c r="C4" s="1" t="inlineStr"/>
+      <c r="D4" s="1" t="inlineStr"/>
+      <c r="E4" s="1" t="inlineStr"/>
+      <c r="F4" s="1" t="inlineStr"/>
+      <c r="G4" s="1" t="inlineStr"/>
+      <c r="H4" s="1" t="inlineStr"/>
     </row>
     <row r="5" ht="12.75" customHeight="1">
-      <c r="A5" t="inlineStr">
+      <c r="A5" s="1" t="inlineStr">
         <is>
           <t>月</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="B5" s="1" t="inlineStr">
         <is>
           <t>担当者</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="C5" s="1" t="inlineStr">
         <is>
           <t>顧客名</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
+      <c r="D5" s="1" t="inlineStr">
         <is>
           <t>案件名</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr">
+      <c r="E5" s="1" t="inlineStr">
         <is>
           <t>売上金額</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr">
+      <c r="F5" s="1" t="inlineStr">
         <is>
           <t>原価</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr">
+      <c r="G5" s="1" t="inlineStr">
         <is>
           <t>粗利</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr">
+      <c r="H5" s="1" t="inlineStr">
         <is>
           <t>粗利率(%)</t>
         </is>
       </c>
     </row>
     <row r="6" ht="12.75" customHeight="1">
-      <c r="A6" t="inlineStr">
+      <c r="A6" s="1" t="inlineStr">
         <is>
           <t>2024/01</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
+      <c r="B6" s="1" t="inlineStr">
         <is>
           <t>田中 一郎</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
+      <c r="C6" s="1" t="inlineStr">
         <is>
           <t>A社</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr">
+      <c r="D6" s="1" t="inlineStr">
         <is>
           <t>システム改修</t>
         </is>
       </c>
-      <c r="E6" t="n">
+      <c r="E6" s="1" t="n">
         <v>800000</v>
       </c>
-      <c r="F6" t="n">
+      <c r="F6" s="1" t="n">
         <v>480000</v>
       </c>
-      <c r="G6" t="n">
+      <c r="G6" s="1" t="n">
         <v>320000</v>
       </c>
-      <c r="H6" t="n">
+      <c r="H6" s="1" t="n">
         <v>40</v>
       </c>
     </row>
     <row r="7" ht="12.75" customHeight="1">
-      <c r="A7" t="inlineStr">
+      <c r="A7" s="1" t="inlineStr">
         <is>
           <t>2024/01</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
+      <c r="B7" s="1" t="inlineStr">
         <is>
           <t>佐藤 二郎</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
+      <c r="C7" s="1" t="inlineStr">
         <is>
           <t>B社</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr">
+      <c r="D7" s="1" t="inlineStr">
         <is>
           <t>コンサルティング</t>
         </is>
       </c>
-      <c r="E7" t="n">
+      <c r="E7" s="1" t="n">
         <v>350000</v>
       </c>
-      <c r="F7" t="n">
+      <c r="F7" s="1" t="n">
         <v>140000</v>
       </c>
-      <c r="G7" t="n">
+      <c r="G7" s="1" t="n">
         <v>210000</v>
       </c>
-      <c r="H7" t="n">
+      <c r="H7" s="1" t="n">
         <v>60</v>
       </c>
     </row>
     <row r="8" ht="12.75" customHeight="1">
-      <c r="A8" t="inlineStr">
+      <c r="A8" s="1" t="inlineStr">
         <is>
           <t>2024/01</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
+      <c r="B8" s="1" t="inlineStr">
         <is>
           <t>鈴木 三郎</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
+      <c r="C8" s="1" t="inlineStr">
         <is>
           <t>C社</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr">
+      <c r="D8" s="1" t="inlineStr">
         <is>
           <t>保守運用</t>
         </is>
       </c>
-      <c r="E8" t="n">
+      <c r="E8" s="1" t="n">
         <v>200000</v>
       </c>
-      <c r="F8" t="n">
+      <c r="F8" s="1" t="n">
         <v>100000</v>
       </c>
-      <c r="G8" t="n">
+      <c r="G8" s="1" t="n">
         <v>100000</v>
       </c>
-      <c r="H8" t="n">
+      <c r="H8" s="1" t="n">
         <v>50</v>
       </c>
     </row>
     <row r="9" ht="12.75" customHeight="1">
-      <c r="A9" t="inlineStr">
+      <c r="A9" s="1" t="inlineStr">
         <is>
           <t>2024/02</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
+      <c r="B9" s="1" t="inlineStr">
         <is>
           <t>田中 一郎</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr">
+      <c r="C9" s="1" t="inlineStr">
         <is>
           <t>D社</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr">
+      <c r="D9" s="1" t="inlineStr">
         <is>
           <t>新規開発</t>
         </is>
       </c>
-      <c r="E9" t="n">
+      <c r="E9" s="1" t="n">
         <v>1200000</v>
       </c>
-      <c r="F9" t="n">
+      <c r="F9" s="1" t="n">
         <v>720000</v>
       </c>
-      <c r="G9" t="n">
+      <c r="G9" s="1" t="n">
         <v>480000</v>
       </c>
-      <c r="H9" t="n">
+      <c r="H9" s="1" t="n">
         <v>40</v>
       </c>
     </row>
     <row r="10" ht="12.75" customHeight="1">
-      <c r="A10" t="inlineStr">
+      <c r="A10" s="1" t="inlineStr">
         <is>
           <t>2024/02</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr">
+      <c r="B10" s="1" t="inlineStr">
         <is>
           <t>佐藤 二郎</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr">
+      <c r="C10" s="1" t="inlineStr">
         <is>
           <t>A社</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr">
+      <c r="D10" s="1" t="inlineStr">
         <is>
           <t>追加開発</t>
         </is>
       </c>
-      <c r="E10" t="n">
+      <c r="E10" s="1" t="n">
         <v>450000</v>
       </c>
-      <c r="F10" t="n">
+      <c r="F10" s="1" t="n">
         <v>225000</v>
       </c>
-      <c r="G10" t="n">
+      <c r="G10" s="1" t="n">
         <v>225000</v>
       </c>
-      <c r="H10" t="n">
+      <c r="H10" s="1" t="n">
         <v>50</v>
       </c>
     </row>
     <row r="11" ht="12.75" customHeight="1">
-      <c r="A11" t="inlineStr">
+      <c r="A11" s="1" t="inlineStr">
         <is>
           <t>2024/02</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr">
+      <c r="B11" s="1" t="inlineStr">
         <is>
           <t>山本 四郎</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr">
+      <c r="C11" s="1" t="inlineStr">
         <is>
           <t>E社</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr">
+      <c r="D11" s="1" t="inlineStr">
         <is>
           <t>システム導入</t>
         </is>
       </c>
-      <c r="E11" t="n">
+      <c r="E11" s="1" t="n">
         <v>600000</v>
       </c>
-      <c r="F11" t="n">
+      <c r="F11" s="1" t="n">
         <v>300000</v>
       </c>
-      <c r="G11" t="n">
+      <c r="G11" s="1" t="n">
         <v>300000</v>
       </c>
-      <c r="H11" t="n">
+      <c r="H11" s="1" t="n">
         <v>50</v>
       </c>
     </row>
     <row r="12" ht="12.75" customHeight="1">
-      <c r="A12" t="inlineStr">
+      <c r="A12" s="1" t="inlineStr">
         <is>
           <t>2024/03</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr">
+      <c r="B12" s="1" t="inlineStr">
         <is>
           <t>田中 一郎</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr">
+      <c r="C12" s="1" t="inlineStr">
         <is>
           <t>F社</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr">
+      <c r="D12" s="1" t="inlineStr">
         <is>
           <t>要件定義</t>
         </is>
       </c>
-      <c r="E12" t="n">
+      <c r="E12" s="1" t="n">
         <v>300000</v>
       </c>
-      <c r="F12" t="n">
+      <c r="F12" s="1" t="n">
         <v>150000</v>
       </c>
-      <c r="G12" t="n">
+      <c r="G12" s="1" t="n">
         <v>150000</v>
       </c>
-      <c r="H12" t="n">
+      <c r="H12" s="1" t="n">
         <v>50</v>
       </c>
     </row>
     <row r="13" ht="12.75" customHeight="1">
-      <c r="A13" t="inlineStr">
+      <c r="A13" s="1" t="inlineStr">
         <is>
           <t>2024/03</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr">
+      <c r="B13" s="1" t="inlineStr">
         <is>
           <t>鈴木 三郎</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr">
+      <c r="C13" s="1" t="inlineStr">
         <is>
           <t>B社</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr">
+      <c r="D13" s="1" t="inlineStr">
         <is>
           <t>テスト支援</t>
         </is>
       </c>
-      <c r="E13" t="n">
+      <c r="E13" s="1" t="n">
         <v>250000</v>
       </c>
-      <c r="F13" t="n">
+      <c r="F13" s="1" t="n">
         <v>125000</v>
       </c>
-      <c r="G13" t="n">
+      <c r="G13" s="1" t="n">
         <v>125000</v>
       </c>
-      <c r="H13" t="n">
+      <c r="H13" s="1" t="n">
         <v>50</v>
       </c>
     </row>
     <row r="14" ht="12.75" customHeight="1">
-      <c r="A14" t="inlineStr">
+      <c r="A14" s="1" t="inlineStr">
         <is>
           <t>2024/03</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr">
+      <c r="B14" s="1" t="inlineStr">
         <is>
           <t>山本 四郎</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr">
+      <c r="C14" s="1" t="inlineStr">
         <is>
           <t>G社</t>
         </is>
       </c>
-      <c r="D14" t="inlineStr">
+      <c r="D14" s="1" t="inlineStr">
         <is>
           <t>インフラ構築</t>
         </is>
       </c>
-      <c r="E14" t="n">
+      <c r="E14" s="1" t="n">
         <v>500000</v>
       </c>
-      <c r="F14" t="n">
+      <c r="F14" s="1" t="n">
         <v>250000</v>
       </c>
-      <c r="G14" t="n">
+      <c r="G14" s="1" t="n">
         <v>250000</v>
       </c>
-      <c r="H14" t="n">
+      <c r="H14" s="1" t="n">
         <v>50</v>
       </c>
     </row>
     <row r="15" ht="12.75" customHeight="1">
-      <c r="A15" t="inlineStr">
+      <c r="A15" s="1" t="inlineStr">
         <is>
           <t>2024/03</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr">
+      <c r="B15" s="1" t="inlineStr">
         <is>
           <t>佐藤 二郎</t>
         </is>
       </c>
-      <c r="C15" t="inlineStr">
+      <c r="C15" s="1" t="inlineStr">
         <is>
           <t>H社</t>
         </is>
       </c>
-      <c r="D15" t="inlineStr">
+      <c r="D15" s="1" t="inlineStr">
         <is>
           <t>運用設計</t>
         </is>
       </c>
-      <c r="E15" t="n">
+      <c r="E15" s="1" t="n">
         <v>380000</v>
       </c>
-      <c r="F15" t="n">
+      <c r="F15" s="1" t="n">
         <v>190000</v>
       </c>
-      <c r="G15" t="n">
+      <c r="G15" s="1" t="n">
         <v>190000</v>
       </c>
-      <c r="H15" t="n">
+      <c r="H15" s="1" t="n">
         <v>50</v>
       </c>
     </row>
     <row r="16" ht="12.75" customHeight="1">
-      <c r="A16" t="inlineStr">
+      <c r="A16" s="1" t="inlineStr">
         <is>
           <t>合計</t>
         </is>
       </c>
-      <c r="B16" t="inlineStr"/>
-      <c r="C16" t="inlineStr"/>
-      <c r="D16" t="inlineStr"/>
-      <c r="E16" t="n">
+      <c r="B16" s="1" t="inlineStr"/>
+      <c r="C16" s="1" t="inlineStr"/>
+      <c r="D16" s="1" t="inlineStr"/>
+      <c r="E16" s="1" t="n">
         <v>5030000</v>
       </c>
-      <c r="F16" t="n">
+      <c r="F16" s="1" t="n">
         <v>2680000</v>
       </c>
-      <c r="G16" t="n">
+      <c r="G16" s="1" t="n">
         <v>2350000</v>
       </c>
-      <c r="H16" t="n">
+      <c r="H16" s="1" t="n">
         <v>49</v>
       </c>
     </row>
     <row r="17">
-      <c r="A17" t="inlineStr"/>
-      <c r="B17" t="inlineStr"/>
-      <c r="C17" t="inlineStr"/>
-      <c r="D17" t="inlineStr"/>
-      <c r="E17" t="inlineStr"/>
-      <c r="F17" t="inlineStr"/>
-      <c r="G17" t="inlineStr"/>
-      <c r="H17" t="inlineStr"/>
+      <c r="A17" s="1" t="inlineStr"/>
+      <c r="B17" s="1" t="inlineStr"/>
+      <c r="C17" s="1" t="inlineStr"/>
+      <c r="D17" s="1" t="inlineStr"/>
+      <c r="E17" s="1" t="inlineStr"/>
+      <c r="F17" s="1" t="inlineStr"/>
+      <c r="G17" s="1" t="inlineStr"/>
+      <c r="H17" s="1" t="inlineStr"/>
     </row>
     <row r="18" ht="12.75" customHeight="1">
-      <c r="A18" t="inlineStr">
+      <c r="A18" s="1" t="inlineStr">
         <is>
           <t>担当者別集計</t>
         </is>
       </c>
-      <c r="B18" t="inlineStr"/>
-      <c r="C18" t="inlineStr"/>
-      <c r="D18" t="inlineStr"/>
-      <c r="E18" t="inlineStr"/>
-      <c r="F18" t="inlineStr"/>
-      <c r="G18" t="inlineStr"/>
-      <c r="H18" t="inlineStr"/>
+      <c r="B18" s="1" t="inlineStr"/>
+      <c r="C18" s="1" t="inlineStr"/>
+      <c r="D18" s="1" t="inlineStr"/>
+      <c r="E18" s="1" t="inlineStr"/>
+      <c r="F18" s="1" t="inlineStr"/>
+      <c r="G18" s="1" t="inlineStr"/>
+      <c r="H18" s="1" t="inlineStr"/>
     </row>
     <row r="19" ht="12.75" customHeight="1">
-      <c r="A19" t="inlineStr">
+      <c r="A19" s="1" t="inlineStr">
         <is>
           <t>担当者</t>
         </is>
       </c>
-      <c r="B19" t="inlineStr">
+      <c r="B19" s="1" t="inlineStr">
         <is>
           <t>売上合計</t>
         </is>
       </c>
-      <c r="C19" t="inlineStr">
+      <c r="C19" s="1" t="inlineStr">
         <is>
           <t>粗利合計</t>
         </is>
       </c>
-      <c r="D19" t="inlineStr"/>
-      <c r="E19" t="inlineStr"/>
-      <c r="F19" t="inlineStr"/>
-      <c r="G19" t="inlineStr"/>
-      <c r="H19" t="inlineStr"/>
+      <c r="D19" s="1" t="inlineStr"/>
+      <c r="E19" s="1" t="inlineStr"/>
+      <c r="F19" s="1" t="inlineStr"/>
+      <c r="G19" s="1" t="inlineStr"/>
+      <c r="H19" s="1" t="inlineStr"/>
     </row>
     <row r="20" ht="12.75" customHeight="1">
-      <c r="A20" t="inlineStr">
+      <c r="A20" s="1" t="inlineStr">
         <is>
           <t>佐藤 二郎</t>
         </is>
       </c>
-      <c r="B20" t="n">
+      <c r="B20" s="1" t="n">
         <v>1180000</v>
       </c>
-      <c r="C20" t="n">
+      <c r="C20" s="1" t="n">
         <v>625000</v>
       </c>
-      <c r="D20" t="inlineStr"/>
-      <c r="E20" t="inlineStr"/>
-      <c r="F20" t="inlineStr"/>
-      <c r="G20" t="inlineStr"/>
-      <c r="H20" t="inlineStr"/>
+      <c r="D20" s="1" t="inlineStr"/>
+      <c r="E20" s="1" t="inlineStr"/>
+      <c r="F20" s="1" t="inlineStr"/>
+      <c r="G20" s="1" t="inlineStr"/>
+      <c r="H20" s="1" t="inlineStr"/>
     </row>
     <row r="21" ht="12.75" customHeight="1">
-      <c r="A21" t="inlineStr">
+      <c r="A21" s="1" t="inlineStr">
         <is>
           <t>山本 四郎</t>
         </is>
       </c>
-      <c r="B21" t="n">
+      <c r="B21" s="1" t="n">
         <v>1100000</v>
       </c>
-      <c r="C21" t="n">
+      <c r="C21" s="1" t="n">
         <v>550000</v>
       </c>
-      <c r="D21" t="inlineStr"/>
-      <c r="E21" t="inlineStr"/>
-      <c r="F21" t="inlineStr"/>
-      <c r="G21" t="inlineStr"/>
-      <c r="H21" t="inlineStr"/>
+      <c r="D21" s="1" t="inlineStr"/>
+      <c r="E21" s="1" t="inlineStr"/>
+      <c r="F21" s="1" t="inlineStr"/>
+      <c r="G21" s="1" t="inlineStr"/>
+      <c r="H21" s="1" t="inlineStr"/>
     </row>
     <row r="22" ht="12.75" customHeight="1">
-      <c r="A22" t="inlineStr">
+      <c r="A22" s="1" t="inlineStr">
         <is>
           <t>田中 一郎</t>
         </is>
       </c>
-      <c r="B22" t="n">
+      <c r="B22" s="1" t="n">
         <v>2300000</v>
       </c>
-      <c r="C22" t="n">
+      <c r="C22" s="1" t="n">
         <v>950000</v>
       </c>
-      <c r="D22" t="inlineStr"/>
-      <c r="E22" t="inlineStr"/>
-      <c r="F22" t="inlineStr"/>
-      <c r="G22" t="inlineStr"/>
-      <c r="H22" t="inlineStr"/>
+      <c r="D22" s="1" t="inlineStr"/>
+      <c r="E22" s="1" t="inlineStr"/>
+      <c r="F22" s="1" t="inlineStr"/>
+      <c r="G22" s="1" t="inlineStr"/>
+      <c r="H22" s="1" t="inlineStr"/>
     </row>
     <row r="23" ht="12.75" customHeight="1">
-      <c r="A23" t="inlineStr">
+      <c r="A23" s="1" t="inlineStr">
         <is>
           <t>鈴木 三郎</t>
         </is>
       </c>
-      <c r="B23" t="n">
+      <c r="B23" s="1" t="n">
         <v>450000</v>
       </c>
-      <c r="C23" t="n">
+      <c r="C23" s="1" t="n">
         <v>225000</v>
       </c>
-      <c r="D23" t="inlineStr"/>
-      <c r="E23" t="inlineStr"/>
-      <c r="F23" t="inlineStr"/>
-      <c r="G23" t="inlineStr"/>
-      <c r="H23" t="inlineStr"/>
+      <c r="D23" s="1" t="inlineStr"/>
+      <c r="E23" s="1" t="inlineStr"/>
+      <c r="F23" s="1" t="inlineStr"/>
+      <c r="G23" s="1" t="inlineStr"/>
+      <c r="H23" s="1" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1515,414 +1519,414 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1" ht="12.75" customHeight="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>経費精算書</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr"/>
-      <c r="C1" t="inlineStr"/>
-      <c r="D1" t="inlineStr"/>
-      <c r="E1" t="inlineStr"/>
-      <c r="F1" t="inlineStr"/>
+      <c r="B1" s="1" t="inlineStr"/>
+      <c r="C1" s="1" t="inlineStr"/>
+      <c r="D1" s="1" t="inlineStr"/>
+      <c r="E1" s="1" t="inlineStr"/>
+      <c r="F1" s="1" t="inlineStr"/>
     </row>
     <row r="2" ht="12.75" customHeight="1">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="1" t="inlineStr">
         <is>
           <t>申請者</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B2" s="1" t="inlineStr">
         <is>
           <t>田中 一郎</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr"/>
-      <c r="D2" t="inlineStr"/>
-      <c r="E2" t="inlineStr"/>
-      <c r="F2" t="inlineStr"/>
+      <c r="C2" s="1" t="inlineStr"/>
+      <c r="D2" s="1" t="inlineStr"/>
+      <c r="E2" s="1" t="inlineStr"/>
+      <c r="F2" s="1" t="inlineStr"/>
     </row>
     <row r="3" ht="12.75" customHeight="1">
-      <c r="A3" t="inlineStr">
+      <c r="A3" s="1" t="inlineStr">
         <is>
           <t>所属</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B3" s="1" t="inlineStr">
         <is>
           <t>開発部 第1グループ</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr"/>
-      <c r="D3" t="inlineStr"/>
-      <c r="E3" t="inlineStr"/>
-      <c r="F3" t="inlineStr"/>
+      <c r="C3" s="1" t="inlineStr"/>
+      <c r="D3" s="1" t="inlineStr"/>
+      <c r="E3" s="1" t="inlineStr"/>
+      <c r="F3" s="1" t="inlineStr"/>
     </row>
     <row r="4" ht="12.75" customHeight="1">
-      <c r="A4" t="inlineStr">
+      <c r="A4" s="1" t="inlineStr">
         <is>
           <t>申請日</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="B4" s="1" t="inlineStr">
         <is>
           <t>2024/03/31</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr"/>
-      <c r="D4" t="inlineStr"/>
-      <c r="E4" t="inlineStr"/>
-      <c r="F4" t="inlineStr"/>
+      <c r="C4" s="1" t="inlineStr"/>
+      <c r="D4" s="1" t="inlineStr"/>
+      <c r="E4" s="1" t="inlineStr"/>
+      <c r="F4" s="1" t="inlineStr"/>
     </row>
     <row r="5" ht="12.75" customHeight="1">
-      <c r="A5" t="inlineStr">
+      <c r="A5" s="1" t="inlineStr">
         <is>
           <t>精算対象月</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="B5" s="1" t="inlineStr">
         <is>
           <t>2024年3月</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr"/>
-      <c r="D5" t="inlineStr"/>
-      <c r="E5" t="inlineStr"/>
-      <c r="F5" t="inlineStr"/>
+      <c r="C5" s="1" t="inlineStr"/>
+      <c r="D5" s="1" t="inlineStr"/>
+      <c r="E5" s="1" t="inlineStr"/>
+      <c r="F5" s="1" t="inlineStr"/>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr"/>
-      <c r="B6" t="inlineStr"/>
-      <c r="C6" t="inlineStr"/>
-      <c r="D6" t="inlineStr"/>
-      <c r="E6" t="inlineStr"/>
-      <c r="F6" t="inlineStr"/>
+      <c r="A6" s="1" t="inlineStr"/>
+      <c r="B6" s="1" t="inlineStr"/>
+      <c r="C6" s="1" t="inlineStr"/>
+      <c r="D6" s="1" t="inlineStr"/>
+      <c r="E6" s="1" t="inlineStr"/>
+      <c r="F6" s="1" t="inlineStr"/>
     </row>
     <row r="7" ht="12.75" customHeight="1">
-      <c r="A7" t="inlineStr">
+      <c r="A7" s="1" t="inlineStr">
         <is>
           <t>日付</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
+      <c r="B7" s="1" t="inlineStr">
         <is>
           <t>費目</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
+      <c r="C7" s="1" t="inlineStr">
         <is>
           <t>内容</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr">
+      <c r="D7" s="1" t="inlineStr">
         <is>
           <t>支払先</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr">
+      <c r="E7" s="1" t="inlineStr">
         <is>
           <t>金額（円）</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr">
+      <c r="F7" s="1" t="inlineStr">
         <is>
           <t>領収書</t>
         </is>
       </c>
     </row>
     <row r="8" ht="12.75" customHeight="1">
-      <c r="A8" t="inlineStr">
+      <c r="A8" s="1" t="inlineStr">
         <is>
           <t>2024/03/05</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
+      <c r="B8" s="1" t="inlineStr">
         <is>
           <t>交通費</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
+      <c r="C8" s="1" t="inlineStr">
         <is>
           <t>客先訪問（A社往復）</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr">
+      <c r="D8" s="1" t="inlineStr">
         <is>
           <t>交通機関</t>
         </is>
       </c>
-      <c r="E8" t="n">
+      <c r="E8" s="1" t="n">
         <v>1640</v>
       </c>
-      <c r="F8" t="inlineStr">
+      <c r="F8" s="1" t="inlineStr">
         <is>
           <t>有</t>
         </is>
       </c>
     </row>
     <row r="9" ht="12.75" customHeight="1">
-      <c r="A9" t="inlineStr">
+      <c r="A9" s="1" t="inlineStr">
         <is>
           <t>2024/03/07</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
+      <c r="B9" s="1" t="inlineStr">
         <is>
           <t>交通費</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr">
+      <c r="C9" s="1" t="inlineStr">
         <is>
           <t>客先訪問（B社往復）</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr">
+      <c r="D9" s="1" t="inlineStr">
         <is>
           <t>交通機関</t>
         </is>
       </c>
-      <c r="E9" t="n">
+      <c r="E9" s="1" t="n">
         <v>2100</v>
       </c>
-      <c r="F9" t="inlineStr">
+      <c r="F9" s="1" t="inlineStr">
         <is>
           <t>有</t>
         </is>
       </c>
     </row>
     <row r="10" ht="12.75" customHeight="1">
-      <c r="A10" t="inlineStr">
+      <c r="A10" s="1" t="inlineStr">
         <is>
           <t>2024/03/12</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr">
+      <c r="B10" s="1" t="inlineStr">
         <is>
           <t>接待費</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr">
+      <c r="C10" s="1" t="inlineStr">
         <is>
           <t>顧客との打合せランチ（3名）</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr">
+      <c r="D10" s="1" t="inlineStr">
         <is>
           <t>〇〇レストラン</t>
         </is>
       </c>
-      <c r="E10" t="n">
+      <c r="E10" s="1" t="n">
         <v>8500</v>
       </c>
-      <c r="F10" t="inlineStr">
+      <c r="F10" s="1" t="inlineStr">
         <is>
           <t>有</t>
         </is>
       </c>
     </row>
     <row r="11" ht="12.75" customHeight="1">
-      <c r="A11" t="inlineStr">
+      <c r="A11" s="1" t="inlineStr">
         <is>
           <t>2024/03/14</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr">
+      <c r="B11" s="1" t="inlineStr">
         <is>
           <t>通信費</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr">
+      <c r="C11" s="1" t="inlineStr">
         <is>
           <t>携帯電話料金（業務分）</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr">
+      <c r="D11" s="1" t="inlineStr">
         <is>
           <t>通信会社</t>
         </is>
       </c>
-      <c r="E11" t="n">
+      <c r="E11" s="1" t="n">
         <v>3000</v>
       </c>
-      <c r="F11" t="inlineStr">
+      <c r="F11" s="1" t="inlineStr">
         <is>
           <t>有</t>
         </is>
       </c>
     </row>
     <row r="12" ht="12.75" customHeight="1">
-      <c r="A12" t="inlineStr">
+      <c r="A12" s="1" t="inlineStr">
         <is>
           <t>2024/03/19</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr">
+      <c r="B12" s="1" t="inlineStr">
         <is>
           <t>交通費</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr">
+      <c r="C12" s="1" t="inlineStr">
         <is>
           <t>セミナー参加（往復）</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr">
+      <c r="D12" s="1" t="inlineStr">
         <is>
           <t>交通機関</t>
         </is>
       </c>
-      <c r="E12" t="n">
+      <c r="E12" s="1" t="n">
         <v>980</v>
       </c>
-      <c r="F12" t="inlineStr">
+      <c r="F12" s="1" t="inlineStr">
         <is>
           <t>有</t>
         </is>
       </c>
     </row>
     <row r="13" ht="12.75" customHeight="1">
-      <c r="A13" t="inlineStr">
+      <c r="A13" s="1" t="inlineStr">
         <is>
           <t>2024/03/19</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr">
+      <c r="B13" s="1" t="inlineStr">
         <is>
           <t>研修費</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr">
+      <c r="C13" s="1" t="inlineStr">
         <is>
           <t>技術セミナー参加費</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr">
+      <c r="D13" s="1" t="inlineStr">
         <is>
           <t>△△協会</t>
         </is>
       </c>
-      <c r="E13" t="n">
+      <c r="E13" s="1" t="n">
         <v>15000</v>
       </c>
-      <c r="F13" t="inlineStr">
+      <c r="F13" s="1" t="inlineStr">
         <is>
           <t>有</t>
         </is>
       </c>
     </row>
     <row r="14" ht="12.75" customHeight="1">
-      <c r="A14" t="inlineStr">
+      <c r="A14" s="1" t="inlineStr">
         <is>
           <t>2024/03/22</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr">
+      <c r="B14" s="1" t="inlineStr">
         <is>
           <t>消耗品費</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr">
+      <c r="C14" s="1" t="inlineStr">
         <is>
           <t>業務用文具・用紙</t>
         </is>
       </c>
-      <c r="D14" t="inlineStr">
+      <c r="D14" s="1" t="inlineStr">
         <is>
           <t>事務用品店</t>
         </is>
       </c>
-      <c r="E14" t="n">
+      <c r="E14" s="1" t="n">
         <v>2350</v>
       </c>
-      <c r="F14" t="inlineStr">
+      <c r="F14" s="1" t="inlineStr">
         <is>
           <t>有</t>
         </is>
       </c>
     </row>
     <row r="15" ht="12.75" customHeight="1">
-      <c r="A15" t="inlineStr">
+      <c r="A15" s="1" t="inlineStr">
         <is>
           <t>2024/03/28</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr">
+      <c r="B15" s="1" t="inlineStr">
         <is>
           <t>交通費</t>
         </is>
       </c>
-      <c r="C15" t="inlineStr">
+      <c r="C15" s="1" t="inlineStr">
         <is>
           <t>月末客先訪問（C社往復）</t>
         </is>
       </c>
-      <c r="D15" t="inlineStr">
+      <c r="D15" s="1" t="inlineStr">
         <is>
           <t>交通機関</t>
         </is>
       </c>
-      <c r="E15" t="n">
+      <c r="E15" s="1" t="n">
         <v>1820</v>
       </c>
-      <c r="F15" t="inlineStr">
+      <c r="F15" s="1" t="inlineStr">
         <is>
           <t>有</t>
         </is>
       </c>
     </row>
     <row r="16" ht="12.75" customHeight="1">
-      <c r="A16" t="inlineStr"/>
-      <c r="B16" t="inlineStr"/>
-      <c r="C16" t="inlineStr"/>
-      <c r="D16" t="inlineStr">
+      <c r="A16" s="1" t="inlineStr"/>
+      <c r="B16" s="1" t="inlineStr"/>
+      <c r="C16" s="1" t="inlineStr"/>
+      <c r="D16" s="1" t="inlineStr">
         <is>
           <t>合計</t>
         </is>
       </c>
-      <c r="E16" t="n">
+      <c r="E16" s="1" t="n">
         <v>35390</v>
       </c>
-      <c r="F16" t="inlineStr"/>
+      <c r="F16" s="1" t="inlineStr"/>
     </row>
     <row r="17">
-      <c r="A17" t="inlineStr"/>
-      <c r="B17" t="inlineStr"/>
-      <c r="C17" t="inlineStr"/>
-      <c r="D17" t="inlineStr"/>
-      <c r="E17" t="inlineStr"/>
-      <c r="F17" t="inlineStr"/>
+      <c r="A17" s="1" t="inlineStr"/>
+      <c r="B17" s="1" t="inlineStr"/>
+      <c r="C17" s="1" t="inlineStr"/>
+      <c r="D17" s="1" t="inlineStr"/>
+      <c r="E17" s="1" t="inlineStr"/>
+      <c r="F17" s="1" t="inlineStr"/>
     </row>
     <row r="18" ht="12.75" customHeight="1">
-      <c r="A18" t="inlineStr">
+      <c r="A18" s="1" t="inlineStr">
         <is>
           <t>承認欄</t>
         </is>
       </c>
-      <c r="B18" t="inlineStr"/>
-      <c r="C18" t="inlineStr"/>
-      <c r="D18" t="inlineStr"/>
-      <c r="E18" t="inlineStr"/>
-      <c r="F18" t="inlineStr"/>
+      <c r="B18" s="1" t="inlineStr"/>
+      <c r="C18" s="1" t="inlineStr"/>
+      <c r="D18" s="1" t="inlineStr"/>
+      <c r="E18" s="1" t="inlineStr"/>
+      <c r="F18" s="1" t="inlineStr"/>
     </row>
     <row r="19" ht="12.75" customHeight="1">
-      <c r="A19" t="inlineStr">
+      <c r="A19" s="1" t="inlineStr">
         <is>
           <t>担当</t>
         </is>
       </c>
-      <c r="B19" t="inlineStr"/>
-      <c r="C19" t="inlineStr">
+      <c r="B19" s="1" t="inlineStr"/>
+      <c r="C19" s="1" t="inlineStr">
         <is>
           <t>課長</t>
         </is>
       </c>
-      <c r="D19" t="inlineStr"/>
-      <c r="E19" t="inlineStr">
+      <c r="D19" s="1" t="inlineStr"/>
+      <c r="E19" s="1" t="inlineStr">
         <is>
           <t>部長</t>
         </is>
       </c>
-      <c r="F19" t="inlineStr"/>
+      <c r="F19" s="1" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>